<commit_message>
Fix sales_attributed view bug and map new stockist C1130
</commit_message>
<xml_diff>
--- a/CFA-Stockist-HQ_Mapping_Master_Updated.xlsx
+++ b/CFA-Stockist-HQ_Mapping_Master_Updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Milind\Desktop\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D102F88F-8C88-4F92-A56D-FEE38FEF4491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F60B8794-7220-451F-9B44-C93F8C3DDC90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="CFA-Stockist-HQ Mapping" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CFA-Stockist-HQ Mapping'!$A$1:$AE$594</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CFA-Stockist-HQ Mapping'!$A$1:$AE$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53609,6 +53609,7 @@
     <row r="629" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="630" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
+  <autoFilter ref="A1:AE1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>